<commit_message>
update capítulo balance materia
Añadido link para descargar Excel de BM MG
</commit_message>
<xml_diff>
--- a/datos/fab_queso_sim.xlsx
+++ b/datos/fab_queso_sim.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/34bf2af71bbc2e43/Documentos/GitHub/master-queseria/website/datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="174" documentId="8_{CF1E59C1-CA92-4C88-887C-A78A793F0426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3644E964-2DFD-4F67-B074-D9B403A8C893}"/>
+  <xr:revisionPtr revIDLastSave="176" documentId="8_{CF1E59C1-CA92-4C88-887C-A78A793F0426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{43653533-5B85-4CD1-86B1-0B3D51C280A4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{3820C6B5-2803-4858-AF88-A2FCB3D2881D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{3820C6B5-2803-4858-AF88-A2FCB3D2881D}"/>
   </bookViews>
   <sheets>
     <sheet name="fab_queso_sim" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="12" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -771,7 +771,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="33" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -806,7 +806,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Énfasis1" xfId="20" builtinId="30" customBuiltin="1"/>
@@ -853,138 +852,33 @@
     <cellStyle name="Título 3" xfId="5" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Total" xfId="18" builtinId="25" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="65">
+  <dxfs count="23">
     <dxf>
-      <alignment vertical="center"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <alignment wrapText="1"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <alignment vertical="center"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <alignment vertical="center"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1028,27 +922,6 @@
     <dxf>
       <alignment vertical="center"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{DADACEEB-7279-4D6E-B5FC-344BE1874627}"/>
@@ -1062,138 +935,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>485775</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4483F406-C1F3-24FE-C1F2-4A88259E960B}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="5048250" y="0"/>
-          <a:ext cx="3533775" cy="3438525"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>323850</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CB8190CB-E522-F2C9-3F3D-4019CB67B890}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="10410825" y="381000"/>
-          <a:ext cx="9410700" cy="3629025"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9709,7 +9450,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DEF4566A-639C-45E8-B56D-71F07FA00779}" name="TablaDinámica1" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" showError="1" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8" rowHeaderCaption="Mes">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DEF4566A-639C-45E8-B56D-71F07FA00779}" name="TablaDinámica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" showError="1" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8" rowHeaderCaption="Mes">
   <location ref="A3:J19" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="32">
     <pivotField numFmtId="14" showAll="0">
@@ -10247,7 +9988,7 @@
     <dataField name="Desviación_x000a_total_x000a_(%)" fld="31" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="14">
-    <format dxfId="57">
+    <format dxfId="22">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="4">
@@ -10259,7 +10000,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="56">
+    <format dxfId="21">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="4">
@@ -10271,7 +10012,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="55">
+    <format dxfId="20">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="4">
@@ -10283,13 +10024,13 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="54">
+    <format dxfId="19">
       <pivotArea field="22" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="53">
+    <format dxfId="18">
       <pivotArea field="22" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="52">
+    <format dxfId="17">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -10298,7 +10039,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="51">
+    <format dxfId="16">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -10307,7 +10048,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="50">
+    <format dxfId="15">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -10316,7 +10057,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="49">
+    <format dxfId="14">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -10325,7 +10066,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="48">
+    <format dxfId="13">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -10334,7 +10075,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="47">
+    <format dxfId="12">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -10343,7 +10084,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="46">
+    <format dxfId="11">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -10352,7 +10093,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="45">
+    <format dxfId="10">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -10361,7 +10102,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="44">
+    <format dxfId="9">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -10387,7 +10128,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4EAA836B-7E28-4F5F-B497-A3F78E114EA5}" name="Tabla2" displayName="Tabla2" ref="A1:T365" totalsRowShown="0">
   <autoFilter ref="A1:T365" xr:uid="{4EAA836B-7E28-4F5F-B497-A3F78E114EA5}"/>
   <tableColumns count="20">
-    <tableColumn id="1" xr3:uid="{0EAAFB95-0462-4A46-895E-2C8949E731AE}" name="fecha" dataDxfId="42"/>
+    <tableColumn id="1" xr3:uid="{0EAAFB95-0462-4A46-895E-2C8949E731AE}" name="fecha" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{B99A55EC-062A-41A1-9987-66C4A77606BA}" name="entrada_kg"/>
     <tableColumn id="3" xr3:uid="{DA11BF6E-5AFF-4E5A-A825-C843AA73522C}" name="entrada_litros"/>
     <tableColumn id="4" xr3:uid="{ED230348-1BB5-43D8-ADE4-81312B15A5A9}" name="entrada_grasa_g_l"/>
@@ -10399,28 +10140,28 @@
     <tableColumn id="10" xr3:uid="{E2106BDF-6A85-4EF5-B55C-0D7CFEBF9BD8}" name="queso_kg"/>
     <tableColumn id="11" xr3:uid="{8A9920A8-F994-40CF-861E-A78626F5DFA0}" name="queso_est_pct"/>
     <tableColumn id="12" xr3:uid="{7BEF460E-C8FD-436F-A522-912A1E3FC0C1}" name="queso_mg_pct"/>
-    <tableColumn id="13" xr3:uid="{4C6E2762-B054-43B2-9A21-BCBED25CD3AE}" name="entrada_grasa_kg" dataDxfId="64">
+    <tableColumn id="13" xr3:uid="{4C6E2762-B054-43B2-9A21-BCBED25CD3AE}" name="entrada_grasa_kg" dataDxfId="7">
       <calculatedColumnFormula>Tabla2[[#This Row],[entrada_litros]]*Tabla2[[#This Row],[entrada_grasa_g_l]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{72F3B23C-8C52-4610-8DE2-F2CFF573C1A3}" name="entrada_prot_kg" dataDxfId="63">
+    <tableColumn id="14" xr3:uid="{72F3B23C-8C52-4610-8DE2-F2CFF573C1A3}" name="entrada_prot_kg" dataDxfId="6">
       <calculatedColumnFormula>Tabla2[[#This Row],[entrada_litros]]*Tabla2[[#This Row],[entrada_prot_g_l]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{1F2FDCA1-AA37-432A-9889-51F7AB1D868E}" name="cuba_fab_grasa_kg" dataDxfId="62">
+    <tableColumn id="15" xr3:uid="{1F2FDCA1-AA37-432A-9889-51F7AB1D868E}" name="cuba_fab_grasa_kg" dataDxfId="5">
       <calculatedColumnFormula>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_grasa_g_l]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{5C5A0D35-AC30-4575-AD36-DFD4AB1AAE78}" name="cuba_fab_prot_kg" dataDxfId="61">
+    <tableColumn id="16" xr3:uid="{5C5A0D35-AC30-4575-AD36-DFD4AB1AAE78}" name="cuba_fab_prot_kg" dataDxfId="4">
       <calculatedColumnFormula>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="20" xr3:uid="{60870160-690E-43AA-BA91-2F2A23C024EA}" name="queso_est_kg" dataDxfId="43">
+    <tableColumn id="20" xr3:uid="{60870160-690E-43AA-BA91-2F2A23C024EA}" name="queso_est_kg" dataDxfId="3">
       <calculatedColumnFormula>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{4D671BF4-2751-4C20-94DC-8DF5C5BD43DC}" name="queso_mg_kg" dataDxfId="60">
+    <tableColumn id="19" xr3:uid="{4D671BF4-2751-4C20-94DC-8DF5C5BD43DC}" name="queso_mg_kg" dataDxfId="2">
       <calculatedColumnFormula>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_mg_pct]]/100</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{557AB84E-05A8-425D-881C-BCA8985A6A4E}" name="semanaISO" dataDxfId="59">
+    <tableColumn id="17" xr3:uid="{557AB84E-05A8-425D-881C-BCA8985A6A4E}" name="semanaISO" dataDxfId="1">
       <calculatedColumnFormula>_xlfn.ISOWEEKNUM(Tabla2[[#This Row],[fecha]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{4C92060C-D738-42A2-A8B9-D53895DE3195}" name="semana" dataDxfId="58"/>
+    <tableColumn id="18" xr3:uid="{4C92060C-D738-42A2-A8B9-D53895DE3195}" name="semana" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -10857,7 +10598,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q2" s="22">
+      <c r="Q2">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -10926,7 +10667,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>180.31849</v>
       </c>
-      <c r="Q3" s="22">
+      <c r="Q3">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>318.86489699999998</v>
       </c>
@@ -10995,7 +10736,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>179.89500000000001</v>
       </c>
-      <c r="Q4" s="22">
+      <c r="Q4">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>302.99867</v>
       </c>
@@ -11064,7 +10805,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>174.00873000000001</v>
       </c>
-      <c r="Q5" s="22">
+      <c r="Q5">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>303.48241499999995</v>
       </c>
@@ -11133,7 +10874,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>176.50821999999999</v>
       </c>
-      <c r="Q6" s="22">
+      <c r="Q6">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>309.06479999999999</v>
       </c>
@@ -11187,7 +10928,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>195.16079999999999</v>
       </c>
-      <c r="Q7" s="22">
+      <c r="Q7">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>340.94821500000006</v>
       </c>
@@ -11223,7 +10964,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q8" s="22">
+      <c r="Q8">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -11274,7 +11015,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q9" s="22">
+      <c r="Q9">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -11343,7 +11084,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>175.8991</v>
       </c>
-      <c r="Q10" s="22">
+      <c r="Q10">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>306.54863700000004</v>
       </c>
@@ -11412,7 +11153,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.35904000000002</v>
       </c>
-      <c r="Q11" s="22">
+      <c r="Q11">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>323.06771200000003</v>
       </c>
@@ -11481,7 +11222,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>175.54939999999999</v>
       </c>
-      <c r="Q12" s="22">
+      <c r="Q12">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>302.49744299999998</v>
       </c>
@@ -11550,7 +11291,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.50129999999999</v>
       </c>
-      <c r="Q13" s="22">
+      <c r="Q13">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>310.48682699999995</v>
       </c>
@@ -11604,7 +11345,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>218.60640000000004</v>
       </c>
-      <c r="Q14" s="22">
+      <c r="Q14">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>387.9083</v>
       </c>
@@ -11640,7 +11381,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q15" s="22">
+      <c r="Q15">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -11691,7 +11432,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q16" s="22">
+      <c r="Q16">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -11760,7 +11501,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>166.74655999999999</v>
       </c>
-      <c r="Q17" s="22">
+      <c r="Q17">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>302.03810399999998</v>
       </c>
@@ -11829,7 +11570,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>168.87325999999999</v>
       </c>
-      <c r="Q18" s="22">
+      <c r="Q18">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>314.90581200000003</v>
       </c>
@@ -11898,7 +11639,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.17689999999999</v>
       </c>
-      <c r="Q19" s="22">
+      <c r="Q19">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>317.22380799999996</v>
       </c>
@@ -11967,7 +11708,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.10843999999997</v>
       </c>
-      <c r="Q20" s="22">
+      <c r="Q20">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>335.71466500000002</v>
       </c>
@@ -12021,7 +11762,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>206.29728</v>
       </c>
-      <c r="Q21" s="22">
+      <c r="Q21">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>375.101856</v>
       </c>
@@ -12057,7 +11798,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q22" s="22">
+      <c r="Q22">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -12108,7 +11849,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q23" s="22">
+      <c r="Q23">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -12177,7 +11918,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.42239999999998</v>
       </c>
-      <c r="Q24" s="22">
+      <c r="Q24">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>300.159108</v>
       </c>
@@ -12246,7 +11987,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>168.68940000000001</v>
       </c>
-      <c r="Q25" s="22">
+      <c r="Q25">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>301.24774400000001</v>
       </c>
@@ -12315,7 +12056,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>174.49126000000001</v>
       </c>
-      <c r="Q26" s="22">
+      <c r="Q26">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>317.54294899999996</v>
       </c>
@@ -12384,7 +12125,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.36416</v>
       </c>
-      <c r="Q27" s="22">
+      <c r="Q27">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>311.991264</v>
       </c>
@@ -12438,7 +12179,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>151.04544999999999</v>
       </c>
-      <c r="Q28" s="22">
+      <c r="Q28">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>261.717848</v>
       </c>
@@ -12474,7 +12215,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q29" s="22">
+      <c r="Q29">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -12525,7 +12266,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q30" s="22">
+      <c r="Q30">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -12594,7 +12335,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>175.80947999999998</v>
       </c>
-      <c r="Q31" s="22">
+      <c r="Q31">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>298.81906399999997</v>
       </c>
@@ -12663,7 +12404,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.73020000000002</v>
       </c>
-      <c r="Q32" s="22">
+      <c r="Q32">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>315.32410499999992</v>
       </c>
@@ -12732,7 +12473,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>175.04014000000001</v>
       </c>
-      <c r="Q33" s="22">
+      <c r="Q33">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>297.84472200000005</v>
       </c>
@@ -12801,7 +12542,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>173.40966</v>
       </c>
-      <c r="Q34" s="22">
+      <c r="Q34">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>309.55273100000005</v>
       </c>
@@ -12855,7 +12596,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>161.05439999999999</v>
       </c>
-      <c r="Q35" s="22">
+      <c r="Q35">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>284.30212599999999</v>
       </c>
@@ -12891,7 +12632,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q36" s="22">
+      <c r="Q36">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -12942,7 +12683,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q37" s="22">
+      <c r="Q37">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -13011,7 +12752,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>167.51705000000001</v>
       </c>
-      <c r="Q38" s="22">
+      <c r="Q38">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>314.20863000000003</v>
       </c>
@@ -13080,7 +12821,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>166.86541999999997</v>
       </c>
-      <c r="Q39" s="22">
+      <c r="Q39">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>318.73766599999993</v>
       </c>
@@ -13149,7 +12890,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>167.6499</v>
       </c>
-      <c r="Q40" s="22">
+      <c r="Q40">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>321.946415</v>
       </c>
@@ -13218,7 +12959,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>167.55101999999999</v>
       </c>
-      <c r="Q41" s="22">
+      <c r="Q41">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>317.640128</v>
       </c>
@@ -13272,7 +13013,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>151.25344000000001</v>
       </c>
-      <c r="Q42" s="22">
+      <c r="Q42">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>275.07363499999997</v>
       </c>
@@ -13308,7 +13049,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q43" s="22">
+      <c r="Q43">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -13359,7 +13100,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q44" s="22">
+      <c r="Q44">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -13428,7 +13169,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>168.01918000000001</v>
       </c>
-      <c r="Q45" s="22">
+      <c r="Q45">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>334.20556199999999</v>
       </c>
@@ -13497,7 +13238,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.80865</v>
       </c>
-      <c r="Q46" s="22">
+      <c r="Q46">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>310.25231500000001</v>
       </c>
@@ -13566,7 +13307,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.44300000000001</v>
       </c>
-      <c r="Q47" s="22">
+      <c r="Q47">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>302.04498000000001</v>
       </c>
@@ -13635,7 +13376,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.82933000000003</v>
       </c>
-      <c r="Q48" s="22">
+      <c r="Q48">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>283.66286400000001</v>
       </c>
@@ -13689,7 +13430,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>243.46751999999998</v>
       </c>
-      <c r="Q49" s="22">
+      <c r="Q49">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>442.04370600000004</v>
       </c>
@@ -13725,7 +13466,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q50" s="22">
+      <c r="Q50">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -13776,7 +13517,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q51" s="22">
+      <c r="Q51">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -13845,7 +13586,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>175.04774000000003</v>
       </c>
-      <c r="Q52" s="22">
+      <c r="Q52">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>294.90070200000002</v>
       </c>
@@ -13914,7 +13655,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>173.46600000000001</v>
       </c>
-      <c r="Q53" s="22">
+      <c r="Q53">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>315.35933000000006</v>
       </c>
@@ -13983,7 +13724,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.178</v>
       </c>
-      <c r="Q54" s="22">
+      <c r="Q54">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>316.13699699999995</v>
       </c>
@@ -14052,7 +13793,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>164.8528</v>
       </c>
-      <c r="Q55" s="22">
+      <c r="Q55">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>286.925276</v>
       </c>
@@ -14106,7 +13847,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>147.19499999999999</v>
       </c>
-      <c r="Q56" s="22">
+      <c r="Q56">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>288.27954</v>
       </c>
@@ -14142,7 +13883,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q57" s="22">
+      <c r="Q57">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -14193,7 +13934,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q58" s="22">
+      <c r="Q58">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -14262,7 +14003,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.95337999999998</v>
       </c>
-      <c r="Q59" s="22">
+      <c r="Q59">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>294.99169799999999</v>
       </c>
@@ -14331,7 +14072,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.03049000000001</v>
       </c>
-      <c r="Q60" s="22">
+      <c r="Q60">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>309.71602200000007</v>
       </c>
@@ -14400,7 +14141,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.41408000000001</v>
       </c>
-      <c r="Q61" s="22">
+      <c r="Q61">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>288.15526999999997</v>
       </c>
@@ -14469,7 +14210,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>168.16996</v>
       </c>
-      <c r="Q62" s="22">
+      <c r="Q62">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>334.80329400000005</v>
       </c>
@@ -14523,7 +14264,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>105.83789</v>
       </c>
-      <c r="Q63" s="22">
+      <c r="Q63">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>209.19094699999997</v>
       </c>
@@ -14559,7 +14300,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q64" s="22">
+      <c r="Q64">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -14610,7 +14351,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q65" s="22">
+      <c r="Q65">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -14679,7 +14420,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>168.48828</v>
       </c>
-      <c r="Q66" s="22">
+      <c r="Q66">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>303.70662799999997</v>
       </c>
@@ -14748,7 +14489,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.37556000000001</v>
       </c>
-      <c r="Q67" s="22">
+      <c r="Q67">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>315.33957000000004</v>
       </c>
@@ -14817,7 +14558,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.1301</v>
       </c>
-      <c r="Q68" s="22">
+      <c r="Q68">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>315.61498499999999</v>
       </c>
@@ -14886,7 +14627,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.31232</v>
       </c>
-      <c r="Q69" s="22">
+      <c r="Q69">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>293.27855999999997</v>
       </c>
@@ -14940,7 +14681,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>141.72543999999999</v>
       </c>
-      <c r="Q70" s="22">
+      <c r="Q70">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>263.03376000000003</v>
       </c>
@@ -14976,7 +14717,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q71" s="22">
+      <c r="Q71">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -15027,7 +14768,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q72" s="22">
+      <c r="Q72">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -15096,7 +14837,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>163.60499999999999</v>
       </c>
-      <c r="Q73" s="22">
+      <c r="Q73">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>318.84832900000004</v>
       </c>
@@ -15165,7 +14906,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>168.75581</v>
       </c>
-      <c r="Q74" s="22">
+      <c r="Q74">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>310.32890900000001</v>
       </c>
@@ -15234,7 +14975,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.11264</v>
       </c>
-      <c r="Q75" s="22">
+      <c r="Q75">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>316.29139200000003</v>
       </c>
@@ -15303,7 +15044,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>166.98074999999997</v>
       </c>
-      <c r="Q76" s="22">
+      <c r="Q76">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>300.22355999999996</v>
       </c>
@@ -15357,7 +15098,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>146.06</v>
       </c>
-      <c r="Q77" s="22">
+      <c r="Q77">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>270.48288300000002</v>
       </c>
@@ -15393,7 +15134,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q78" s="22">
+      <c r="Q78">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -15444,7 +15185,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q79" s="22">
+      <c r="Q79">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -15513,7 +15254,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.79556000000002</v>
       </c>
-      <c r="Q80" s="22">
+      <c r="Q80">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>301.451414</v>
       </c>
@@ -15582,7 +15323,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.4727</v>
       </c>
-      <c r="Q81" s="22">
+      <c r="Q81">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>296.86415</v>
       </c>
@@ -15651,7 +15392,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.31381999999996</v>
       </c>
-      <c r="Q82" s="22">
+      <c r="Q82">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>308.43467200000003</v>
       </c>
@@ -15720,7 +15461,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>174.49069999999998</v>
       </c>
-      <c r="Q83" s="22">
+      <c r="Q83">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>298.36753100000004</v>
       </c>
@@ -15774,7 +15515,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>153.72756000000001</v>
       </c>
-      <c r="Q84" s="22">
+      <c r="Q84">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>270.88812000000001</v>
       </c>
@@ -15810,7 +15551,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q85" s="22">
+      <c r="Q85">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -15861,7 +15602,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q86" s="22">
+      <c r="Q86">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -15930,7 +15671,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.13579999999999</v>
       </c>
-      <c r="Q87" s="22">
+      <c r="Q87">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>290.859486</v>
       </c>
@@ -15999,7 +15740,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.93425999999997</v>
       </c>
-      <c r="Q88" s="22">
+      <c r="Q88">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>317.27373599999999</v>
       </c>
@@ -16068,7 +15809,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.36609999999999</v>
       </c>
-      <c r="Q89" s="22">
+      <c r="Q89">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>310.67391499999997</v>
       </c>
@@ -16137,7 +15878,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>173.63560000000001</v>
       </c>
-      <c r="Q90" s="22">
+      <c r="Q90">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>293.33331000000004</v>
       </c>
@@ -16191,7 +15932,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>200.35544999999999</v>
       </c>
-      <c r="Q91" s="22">
+      <c r="Q91">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>336.59479200000004</v>
       </c>
@@ -16227,7 +15968,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q92" s="22">
+      <c r="Q92">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -16278,7 +16019,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q93" s="22">
+      <c r="Q93">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -16347,7 +16088,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.36252999999999</v>
       </c>
-      <c r="Q94" s="22">
+      <c r="Q94">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>287.95120200000002</v>
       </c>
@@ -16416,7 +16157,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.82854</v>
       </c>
-      <c r="Q95" s="22">
+      <c r="Q95">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>313.23394199999996</v>
       </c>
@@ -16485,7 +16226,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.85</v>
       </c>
-      <c r="Q96" s="22">
+      <c r="Q96">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>326.22625599999998</v>
       </c>
@@ -16554,7 +16295,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>168.78941999999998</v>
       </c>
-      <c r="Q97" s="22">
+      <c r="Q97">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>296.52183599999995</v>
       </c>
@@ -16608,7 +16349,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>167.69254000000001</v>
       </c>
-      <c r="Q98" s="22">
+      <c r="Q98">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>291.36320799999999</v>
       </c>
@@ -16644,7 +16385,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q99" s="22">
+      <c r="Q99">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -16695,7 +16436,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q100" s="22">
+      <c r="Q100">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -16764,7 +16505,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.59443999999996</v>
       </c>
-      <c r="Q101" s="22">
+      <c r="Q101">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>307.77028799999994</v>
       </c>
@@ -16833,7 +16574,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.53217999999998</v>
       </c>
-      <c r="Q102" s="22">
+      <c r="Q102">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>308.00425000000001</v>
       </c>
@@ -16902,7 +16643,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.81861999999998</v>
       </c>
-      <c r="Q103" s="22">
+      <c r="Q103">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>327.85602</v>
       </c>
@@ -16971,7 +16712,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.054</v>
       </c>
-      <c r="Q104" s="22">
+      <c r="Q104">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>292.68566400000003</v>
       </c>
@@ -17025,7 +16766,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>125.03988000000001</v>
       </c>
-      <c r="Q105" s="22">
+      <c r="Q105">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>234.19096399999998</v>
       </c>
@@ -17061,7 +16802,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q106" s="22">
+      <c r="Q106">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -17112,7 +16853,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q107" s="22">
+      <c r="Q107">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -17181,7 +16922,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.80120000000002</v>
       </c>
-      <c r="Q108" s="22">
+      <c r="Q108">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>302.98919799999999</v>
       </c>
@@ -17250,7 +16991,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>175.28310999999999</v>
       </c>
-      <c r="Q109" s="22">
+      <c r="Q109">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>319.52921200000003</v>
       </c>
@@ -17319,7 +17060,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.72231999999997</v>
       </c>
-      <c r="Q110" s="22">
+      <c r="Q110">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>301.69026400000001</v>
       </c>
@@ -17388,7 +17129,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.98599999999999</v>
       </c>
-      <c r="Q111" s="22">
+      <c r="Q111">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>313.08353999999997</v>
       </c>
@@ -17442,7 +17183,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.82363999999998</v>
       </c>
-      <c r="Q112" s="22">
+      <c r="Q112">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>292.87780200000003</v>
       </c>
@@ -17478,7 +17219,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q113" s="22">
+      <c r="Q113">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -17529,7 +17270,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q114" s="22">
+      <c r="Q114">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -17598,7 +17339,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>168.85569999999998</v>
       </c>
-      <c r="Q115" s="22">
+      <c r="Q115">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>300.35292800000002</v>
       </c>
@@ -17667,7 +17408,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>177.69319000000002</v>
       </c>
-      <c r="Q116" s="22">
+      <c r="Q116">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>314.060205</v>
       </c>
@@ -17736,7 +17477,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>176.9051</v>
       </c>
-      <c r="Q117" s="22">
+      <c r="Q117">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>302.50019800000001</v>
       </c>
@@ -17805,7 +17546,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>178.9171</v>
       </c>
-      <c r="Q118" s="22">
+      <c r="Q118">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>328.36831999999993</v>
       </c>
@@ -17859,7 +17600,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>164.99231</v>
       </c>
-      <c r="Q119" s="22">
+      <c r="Q119">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>288.52091999999999</v>
       </c>
@@ -17895,7 +17636,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q120" s="22">
+      <c r="Q120">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -17946,7 +17687,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q121" s="22">
+      <c r="Q121">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -18015,7 +17756,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>179.15583999999998</v>
       </c>
-      <c r="Q122" s="22">
+      <c r="Q122">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>311.041696</v>
       </c>
@@ -18084,7 +17825,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>174.44039999999998</v>
       </c>
-      <c r="Q123" s="22">
+      <c r="Q123">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>297.69246399999997</v>
       </c>
@@ -18153,7 +17894,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.06126999999998</v>
       </c>
-      <c r="Q124" s="22">
+      <c r="Q124">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>309.94915999999995</v>
       </c>
@@ -18222,7 +17963,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.88090000000003</v>
       </c>
-      <c r="Q125" s="22">
+      <c r="Q125">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>310.87559999999996</v>
       </c>
@@ -18276,7 +18017,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>192.60300000000001</v>
       </c>
-      <c r="Q126" s="22">
+      <c r="Q126">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>365.25035699999995</v>
       </c>
@@ -18312,7 +18053,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q127" s="22">
+      <c r="Q127">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -18363,7 +18104,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q128" s="22">
+      <c r="Q128">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -18432,7 +18173,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.59759999999997</v>
       </c>
-      <c r="Q129" s="22">
+      <c r="Q129">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>306.22107999999997</v>
       </c>
@@ -18501,7 +18242,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>176.53779</v>
       </c>
-      <c r="Q130" s="22">
+      <c r="Q130">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>318.83238</v>
       </c>
@@ -18570,7 +18311,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.41848000000002</v>
       </c>
-      <c r="Q131" s="22">
+      <c r="Q131">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>303.02731799999998</v>
       </c>
@@ -18639,7 +18380,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>173.26488000000001</v>
       </c>
-      <c r="Q132" s="22">
+      <c r="Q132">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>305.37106899999998</v>
       </c>
@@ -18693,7 +18434,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>179.77782000000002</v>
       </c>
-      <c r="Q133" s="22">
+      <c r="Q133">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>329.75341000000003</v>
       </c>
@@ -18729,7 +18470,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q134" s="22">
+      <c r="Q134">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -18780,7 +18521,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q135" s="22">
+      <c r="Q135">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -18849,7 +18590,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>175.23712000000003</v>
       </c>
-      <c r="Q136" s="22">
+      <c r="Q136">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>296.824164</v>
       </c>
@@ -18918,7 +18659,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.15415999999999</v>
       </c>
-      <c r="Q137" s="22">
+      <c r="Q137">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>299.05250100000006</v>
       </c>
@@ -18987,7 +18728,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.94150999999999</v>
       </c>
-      <c r="Q138" s="22">
+      <c r="Q138">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>307.88596799999999</v>
       </c>
@@ -19056,7 +18797,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.14122</v>
       </c>
-      <c r="Q139" s="22">
+      <c r="Q139">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>303.34414500000003</v>
       </c>
@@ -19110,7 +18851,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.56128000000001</v>
       </c>
-      <c r="Q140" s="22">
+      <c r="Q140">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>308.54831799999999</v>
       </c>
@@ -19146,7 +18887,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q141" s="22">
+      <c r="Q141">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -19197,7 +18938,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q142" s="22">
+      <c r="Q142">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -19266,7 +19007,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.82854</v>
       </c>
-      <c r="Q143" s="22">
+      <c r="Q143">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>306.58225000000004</v>
       </c>
@@ -19335,7 +19076,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.92919000000001</v>
       </c>
-      <c r="Q144" s="22">
+      <c r="Q144">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>312.31288699999999</v>
       </c>
@@ -19404,7 +19145,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.60564000000002</v>
       </c>
-      <c r="Q145" s="22">
+      <c r="Q145">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>311.39461000000006</v>
       </c>
@@ -19473,7 +19214,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>167.91865999999999</v>
       </c>
-      <c r="Q146" s="22">
+      <c r="Q146">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>314.11743000000001</v>
       </c>
@@ -19527,7 +19268,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>148.73088000000001</v>
       </c>
-      <c r="Q147" s="22">
+      <c r="Q147">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>273.32406599999996</v>
       </c>
@@ -19563,7 +19304,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q148" s="22">
+      <c r="Q148">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -19614,7 +19355,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q149" s="22">
+      <c r="Q149">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -19683,7 +19424,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.00685999999999</v>
       </c>
-      <c r="Q150" s="22">
+      <c r="Q150">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>337.90796999999998</v>
       </c>
@@ -19752,7 +19493,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.19219999999999</v>
       </c>
-      <c r="Q151" s="22">
+      <c r="Q151">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>322.50765000000001</v>
       </c>
@@ -19821,7 +19562,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.649</v>
       </c>
-      <c r="Q152" s="22">
+      <c r="Q152">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>319.82082600000001</v>
       </c>
@@ -19890,7 +19631,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.64400000000001</v>
       </c>
-      <c r="Q153" s="22">
+      <c r="Q153">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>321.52760999999998</v>
       </c>
@@ -19944,7 +19685,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>156.5095</v>
       </c>
-      <c r="Q154" s="22">
+      <c r="Q154">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>285.04331399999995</v>
       </c>
@@ -19980,7 +19721,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q155" s="22">
+      <c r="Q155">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -20031,7 +19772,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q156" s="22">
+      <c r="Q156">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -20100,7 +19841,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.16398000000001</v>
       </c>
-      <c r="Q157" s="22">
+      <c r="Q157">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>298.570761</v>
       </c>
@@ -20169,7 +19910,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.54257999999999</v>
       </c>
-      <c r="Q158" s="22">
+      <c r="Q158">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>318.57291900000001</v>
       </c>
@@ -20238,7 +19979,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.48061999999999</v>
       </c>
-      <c r="Q159" s="22">
+      <c r="Q159">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>317.40009599999996</v>
       </c>
@@ -20307,7 +20048,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>175.47300000000001</v>
       </c>
-      <c r="Q160" s="22">
+      <c r="Q160">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>313.74223999999992</v>
       </c>
@@ -20361,7 +20102,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>154.73339999999999</v>
       </c>
-      <c r="Q161" s="22">
+      <c r="Q161">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>266.07095999999996</v>
       </c>
@@ -20397,7 +20138,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q162" s="22">
+      <c r="Q162">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -20448,7 +20189,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q163" s="22">
+      <c r="Q163">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -20517,7 +20258,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>175.35714000000002</v>
       </c>
-      <c r="Q164" s="22">
+      <c r="Q164">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>307.95287500000001</v>
       </c>
@@ -20586,7 +20327,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.15890000000002</v>
       </c>
-      <c r="Q165" s="22">
+      <c r="Q165">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>321.44712599999997</v>
       </c>
@@ -20655,7 +20396,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>164.68451999999999</v>
       </c>
-      <c r="Q166" s="22">
+      <c r="Q166">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>308.85596599999997</v>
       </c>
@@ -20724,7 +20465,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>165.79342000000003</v>
       </c>
-      <c r="Q167" s="22">
+      <c r="Q167">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>338.94638500000002</v>
       </c>
@@ -20778,7 +20519,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>190.51626999999999</v>
       </c>
-      <c r="Q168" s="22">
+      <c r="Q168">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>348.69437100000005</v>
       </c>
@@ -20814,7 +20555,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q169" s="22">
+      <c r="Q169">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -20865,7 +20606,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q170" s="22">
+      <c r="Q170">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -20934,7 +20675,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.70392999999999</v>
       </c>
-      <c r="Q171" s="22">
+      <c r="Q171">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>327.47180399999996</v>
       </c>
@@ -21003,7 +20744,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>176.07132000000001</v>
       </c>
-      <c r="Q172" s="22">
+      <c r="Q172">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>312.16477800000001</v>
       </c>
@@ -21072,7 +20813,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>179.22167999999999</v>
       </c>
-      <c r="Q173" s="22">
+      <c r="Q173">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>313.50006299999995</v>
       </c>
@@ -21141,7 +20882,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>174.76485</v>
       </c>
-      <c r="Q174" s="22">
+      <c r="Q174">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>317.39630400000004</v>
       </c>
@@ -21195,7 +20936,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>196.80627999999999</v>
       </c>
-      <c r="Q175" s="22">
+      <c r="Q175">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>343.51996200000002</v>
       </c>
@@ -21231,7 +20972,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q176" s="22">
+      <c r="Q176">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -21282,7 +21023,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q177" s="22">
+      <c r="Q177">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -21351,7 +21092,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.69998999999999</v>
       </c>
-      <c r="Q178" s="22">
+      <c r="Q178">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>309.45499999999998</v>
       </c>
@@ -21420,7 +21161,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.6378</v>
       </c>
-      <c r="Q179" s="22">
+      <c r="Q179">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>306.20133999999996</v>
       </c>
@@ -21489,7 +21230,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.72874999999999</v>
       </c>
-      <c r="Q180" s="22">
+      <c r="Q180">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>291.87752</v>
       </c>
@@ -21558,7 +21299,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.17599999999999</v>
       </c>
-      <c r="Q181" s="22">
+      <c r="Q181">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>316.76142700000003</v>
       </c>
@@ -21612,7 +21353,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.05929999999998</v>
       </c>
-      <c r="Q182" s="22">
+      <c r="Q182">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>311.33459500000004</v>
       </c>
@@ -21648,7 +21389,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q183" s="22">
+      <c r="Q183">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -21699,7 +21440,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q184" s="22">
+      <c r="Q184">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -21768,7 +21509,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.01314000000002</v>
       </c>
-      <c r="Q185" s="22">
+      <c r="Q185">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>299.47505000000001</v>
       </c>
@@ -21837,7 +21578,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.99909999999997</v>
       </c>
-      <c r="Q186" s="22">
+      <c r="Q186">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>314.20612</v>
       </c>
@@ -21906,7 +21647,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>174.73079999999999</v>
       </c>
-      <c r="Q187" s="22">
+      <c r="Q187">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>304.83221000000003</v>
       </c>
@@ -21975,7 +21716,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>166.77975000000001</v>
       </c>
-      <c r="Q188" s="22">
+      <c r="Q188">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>320.312592</v>
       </c>
@@ -22029,7 +21770,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>162.32433</v>
       </c>
-      <c r="Q189" s="22">
+      <c r="Q189">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>309.05207999999999</v>
       </c>
@@ -22065,7 +21806,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q190" s="22">
+      <c r="Q190">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -22116,7 +21857,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q191" s="22">
+      <c r="Q191">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -22185,7 +21926,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.15890000000002</v>
       </c>
-      <c r="Q192" s="22">
+      <c r="Q192">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>318.47215999999997</v>
       </c>
@@ -22254,7 +21995,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.48712</v>
       </c>
-      <c r="Q193" s="22">
+      <c r="Q193">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>315.36050399999999</v>
       </c>
@@ -22323,7 +22064,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.9194</v>
       </c>
-      <c r="Q194" s="22">
+      <c r="Q194">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>299.19847100000004</v>
       </c>
@@ -22392,7 +22133,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>175.93583999999998</v>
       </c>
-      <c r="Q195" s="22">
+      <c r="Q195">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>295.8279</v>
       </c>
@@ -22446,7 +22187,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>221.91932</v>
       </c>
-      <c r="Q196" s="22">
+      <c r="Q196">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>377.85504500000002</v>
       </c>
@@ -22482,7 +22223,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q197" s="22">
+      <c r="Q197">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -22533,7 +22274,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q198" s="22">
+      <c r="Q198">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -22602,7 +22343,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>177.84960000000001</v>
       </c>
-      <c r="Q199" s="22">
+      <c r="Q199">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>323.13403200000005</v>
       </c>
@@ -22671,7 +22412,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>173.62266</v>
       </c>
-      <c r="Q200" s="22">
+      <c r="Q200">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>303.45249000000001</v>
       </c>
@@ -22740,7 +22481,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>173.86163999999999</v>
       </c>
-      <c r="Q201" s="22">
+      <c r="Q201">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>310.69316400000002</v>
       </c>
@@ -22809,7 +22550,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>177.1354</v>
       </c>
-      <c r="Q202" s="22">
+      <c r="Q202">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>302.68035200000003</v>
       </c>
@@ -22863,7 +22604,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>214.53233999999998</v>
       </c>
-      <c r="Q203" s="22">
+      <c r="Q203">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>386.59868799999998</v>
       </c>
@@ -22899,7 +22640,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q204" s="22">
+      <c r="Q204">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -22950,7 +22691,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q205" s="22">
+      <c r="Q205">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -23019,7 +22760,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.23061999999999</v>
       </c>
-      <c r="Q206" s="22">
+      <c r="Q206">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>299.51009999999997</v>
       </c>
@@ -23088,7 +22829,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>168.78995999999998</v>
       </c>
-      <c r="Q207" s="22">
+      <c r="Q207">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>298.11462399999999</v>
       </c>
@@ -23157,7 +22898,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.20175</v>
       </c>
-      <c r="Q208" s="22">
+      <c r="Q208">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>309.64164</v>
       </c>
@@ -23226,7 +22967,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.45548000000002</v>
       </c>
-      <c r="Q209" s="22">
+      <c r="Q209">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>300.23495100000002</v>
       </c>
@@ -23280,7 +23021,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>157.97475</v>
       </c>
-      <c r="Q210" s="22">
+      <c r="Q210">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>276.98101200000002</v>
       </c>
@@ -23316,7 +23057,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q211" s="22">
+      <c r="Q211">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -23367,7 +23108,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q212" s="22">
+      <c r="Q212">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -23436,7 +23177,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.60906000000003</v>
       </c>
-      <c r="Q213" s="22">
+      <c r="Q213">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>304.974917</v>
       </c>
@@ -23505,7 +23246,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.35249999999999</v>
       </c>
-      <c r="Q214" s="22">
+      <c r="Q214">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>320.44930399999998</v>
       </c>
@@ -23574,7 +23315,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.18299999999999</v>
       </c>
-      <c r="Q215" s="22">
+      <c r="Q215">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>313.26455999999996</v>
       </c>
@@ -23643,7 +23384,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>167.65045000000001</v>
       </c>
-      <c r="Q216" s="22">
+      <c r="Q216">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>299.29727200000002</v>
       </c>
@@ -23697,7 +23438,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>157.22854000000001</v>
       </c>
-      <c r="Q217" s="22">
+      <c r="Q217">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>283.72100400000005</v>
       </c>
@@ -23733,7 +23474,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q218" s="22">
+      <c r="Q218">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -23784,7 +23525,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q219" s="22">
+      <c r="Q219">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -23853,7 +23594,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.72716999999997</v>
       </c>
-      <c r="Q220" s="22">
+      <c r="Q220">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>295.400105</v>
       </c>
@@ -23922,7 +23663,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.67775999999998</v>
       </c>
-      <c r="Q221" s="22">
+      <c r="Q221">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>308.75949800000001</v>
       </c>
@@ -23991,7 +23732,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.14975999999999</v>
       </c>
-      <c r="Q222" s="22">
+      <c r="Q222">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>302.63360399999999</v>
       </c>
@@ -24060,7 +23801,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.00369000000001</v>
       </c>
-      <c r="Q223" s="22">
+      <c r="Q223">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>312.468052</v>
       </c>
@@ -24114,7 +23855,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>108.25794</v>
       </c>
-      <c r="Q224" s="22">
+      <c r="Q224">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>184.27872599999998</v>
       </c>
@@ -24150,7 +23891,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q225" s="22">
+      <c r="Q225">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -24201,7 +23942,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q226" s="22">
+      <c r="Q226">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -24270,7 +24011,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>173.4315</v>
       </c>
-      <c r="Q227" s="22">
+      <c r="Q227">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>329.16177499999998</v>
       </c>
@@ -24339,7 +24080,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.93946</v>
       </c>
-      <c r="Q228" s="22">
+      <c r="Q228">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>299.00382000000002</v>
       </c>
@@ -24408,7 +24149,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>168.42099999999999</v>
       </c>
-      <c r="Q229" s="22">
+      <c r="Q229">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>303.27670200000006</v>
       </c>
@@ -24477,7 +24218,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.91667999999999</v>
       </c>
-      <c r="Q230" s="22">
+      <c r="Q230">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>305.970372</v>
       </c>
@@ -24531,7 +24272,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.22248000000002</v>
       </c>
-      <c r="Q231" s="22">
+      <c r="Q231">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>312.59525400000001</v>
       </c>
@@ -24567,7 +24308,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q232" s="22">
+      <c r="Q232">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -24618,7 +24359,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q233" s="22">
+      <c r="Q233">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -24687,7 +24428,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.46039999999999</v>
       </c>
-      <c r="Q234" s="22">
+      <c r="Q234">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>312.41502600000001</v>
       </c>
@@ -24756,7 +24497,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.56960000000001</v>
       </c>
-      <c r="Q235" s="22">
+      <c r="Q235">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>314.11389600000001</v>
       </c>
@@ -24825,7 +24566,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>167.8186</v>
       </c>
-      <c r="Q236" s="22">
+      <c r="Q236">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>287.62047999999999</v>
       </c>
@@ -24894,7 +24635,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>168.97372000000001</v>
       </c>
-      <c r="Q237" s="22">
+      <c r="Q237">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>297.73619400000001</v>
       </c>
@@ -24948,7 +24689,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>159.54906</v>
       </c>
-      <c r="Q238" s="22">
+      <c r="Q238">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>291.796469</v>
       </c>
@@ -24984,7 +24725,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q239" s="22">
+      <c r="Q239">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -25035,7 +24776,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q240" s="22">
+      <c r="Q240">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -25104,7 +24845,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.6378</v>
       </c>
-      <c r="Q241" s="22">
+      <c r="Q241">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>312.50692000000004</v>
       </c>
@@ -25173,7 +24914,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.78040000000001</v>
       </c>
-      <c r="Q242" s="22">
+      <c r="Q242">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>303.58561200000003</v>
       </c>
@@ -25242,7 +24983,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.71072000000001</v>
       </c>
-      <c r="Q243" s="22">
+      <c r="Q243">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>319.58390100000003</v>
       </c>
@@ -25311,7 +25052,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.53918999999999</v>
       </c>
-      <c r="Q244" s="22">
+      <c r="Q244">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>299.30115599999999</v>
       </c>
@@ -25365,7 +25106,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>153.89419000000001</v>
       </c>
-      <c r="Q245" s="22">
+      <c r="Q245">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>277.41475499999996</v>
       </c>
@@ -25401,7 +25142,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q246" s="22">
+      <c r="Q246">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -25452,7 +25193,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q247" s="22">
+      <c r="Q247">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -25521,7 +25262,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>166.34464</v>
       </c>
-      <c r="Q248" s="22">
+      <c r="Q248">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>314.025464</v>
       </c>
@@ -25590,7 +25331,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.99668000000003</v>
       </c>
-      <c r="Q249" s="22">
+      <c r="Q249">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>290.327832</v>
       </c>
@@ -25659,7 +25400,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.19296000000003</v>
       </c>
-      <c r="Q250" s="22">
+      <c r="Q250">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>299.44028400000002</v>
       </c>
@@ -25728,7 +25469,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.39774999999997</v>
       </c>
-      <c r="Q251" s="22">
+      <c r="Q251">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>331.02339199999994</v>
       </c>
@@ -25782,7 +25523,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>130.02170999999998</v>
       </c>
-      <c r="Q252" s="22">
+      <c r="Q252">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>229.90438399999999</v>
       </c>
@@ -25818,7 +25559,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q253" s="22">
+      <c r="Q253">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -25869,7 +25610,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q254" s="22">
+      <c r="Q254">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -25938,7 +25679,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>177.54816</v>
       </c>
-      <c r="Q255" s="22">
+      <c r="Q255">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>301.258152</v>
       </c>
@@ -26007,7 +25748,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>173.80224000000001</v>
       </c>
-      <c r="Q256" s="22">
+      <c r="Q256">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>276.231177</v>
       </c>
@@ -26076,7 +25817,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>176.60329999999999</v>
       </c>
-      <c r="Q257" s="22">
+      <c r="Q257">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>309.497409</v>
       </c>
@@ -26145,7 +25886,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.67487999999997</v>
       </c>
-      <c r="Q258" s="22">
+      <c r="Q258">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>316.40519999999998</v>
       </c>
@@ -26199,7 +25940,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>160.67250000000001</v>
       </c>
-      <c r="Q259" s="22">
+      <c r="Q259">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>287.25763000000001</v>
       </c>
@@ -26235,7 +25976,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q260" s="22">
+      <c r="Q260">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -26286,7 +26027,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q261" s="22">
+      <c r="Q261">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -26355,7 +26096,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.5744</v>
       </c>
-      <c r="Q262" s="22">
+      <c r="Q262">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>329.38151499999998</v>
       </c>
@@ -26424,7 +26165,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>167.73479999999998</v>
       </c>
-      <c r="Q263" s="22">
+      <c r="Q263">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>312.21372999999994</v>
       </c>
@@ -26493,7 +26234,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.09074000000001</v>
       </c>
-      <c r="Q264" s="22">
+      <c r="Q264">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>309.57350400000001</v>
       </c>
@@ -26562,7 +26303,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>165.55644000000001</v>
       </c>
-      <c r="Q265" s="22">
+      <c r="Q265">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>310.18302</v>
       </c>
@@ -26616,7 +26357,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.81107</v>
       </c>
-      <c r="Q266" s="22">
+      <c r="Q266">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>329.28043000000002</v>
       </c>
@@ -26652,7 +26393,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q267" s="22">
+      <c r="Q267">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -26703,7 +26444,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q268" s="22">
+      <c r="Q268">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -26772,7 +26513,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.61098000000001</v>
       </c>
-      <c r="Q269" s="22">
+      <c r="Q269">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>314.02285499999994</v>
       </c>
@@ -26841,7 +26582,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>173.28718000000001</v>
       </c>
-      <c r="Q270" s="22">
+      <c r="Q270">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>322.19748599999997</v>
       </c>
@@ -26910,7 +26651,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.91167999999999</v>
       </c>
-      <c r="Q271" s="22">
+      <c r="Q271">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>301.44945600000005</v>
       </c>
@@ -26979,7 +26720,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.35833</v>
       </c>
-      <c r="Q272" s="22">
+      <c r="Q272">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>313.85619999999994</v>
       </c>
@@ -27033,7 +26774,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>191.59140000000002</v>
       </c>
-      <c r="Q273" s="22">
+      <c r="Q273">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>357.03544499999998</v>
       </c>
@@ -27069,7 +26810,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q274" s="22">
+      <c r="Q274">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -27120,7 +26861,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q275" s="22">
+      <c r="Q275">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -27189,7 +26930,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>173.72660000000002</v>
       </c>
-      <c r="Q276" s="22">
+      <c r="Q276">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>302.10578300000003</v>
       </c>
@@ -27258,7 +26999,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>166.91499999999999</v>
       </c>
-      <c r="Q277" s="22">
+      <c r="Q277">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>297.47307799999999</v>
       </c>
@@ -27327,7 +27068,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.00623999999999</v>
       </c>
-      <c r="Q278" s="22">
+      <c r="Q278">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>304.56160899999998</v>
       </c>
@@ -27396,7 +27137,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.86624</v>
       </c>
-      <c r="Q279" s="22">
+      <c r="Q279">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>313.36451299999999</v>
       </c>
@@ -27450,7 +27191,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>175.9632</v>
       </c>
-      <c r="Q280" s="22">
+      <c r="Q280">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>326.14987500000001</v>
       </c>
@@ -27486,7 +27227,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q281" s="22">
+      <c r="Q281">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -27537,7 +27278,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q282" s="22">
+      <c r="Q282">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -27606,7 +27347,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.71692000000002</v>
       </c>
-      <c r="Q283" s="22">
+      <c r="Q283">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>320.98411800000002</v>
       </c>
@@ -27675,7 +27416,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>168.52178000000001</v>
       </c>
-      <c r="Q284" s="22">
+      <c r="Q284">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>310.49340999999998</v>
       </c>
@@ -27744,7 +27485,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.58140000000003</v>
       </c>
-      <c r="Q285" s="22">
+      <c r="Q285">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>306.38069999999999</v>
       </c>
@@ -27813,7 +27554,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>164.65175999999997</v>
       </c>
-      <c r="Q286" s="22">
+      <c r="Q286">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>307.72818000000001</v>
       </c>
@@ -27867,7 +27608,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>163.78752000000003</v>
       </c>
-      <c r="Q287" s="22">
+      <c r="Q287">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>310.44822600000003</v>
       </c>
@@ -27903,7 +27644,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q288" s="22">
+      <c r="Q288">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -27954,7 +27695,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q289" s="22">
+      <c r="Q289">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -28023,7 +27764,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>174.33056999999999</v>
       </c>
-      <c r="Q290" s="22">
+      <c r="Q290">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>309.07903800000003</v>
       </c>
@@ -28092,7 +27833,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>176.54336000000001</v>
       </c>
-      <c r="Q291" s="22">
+      <c r="Q291">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>313.19079999999997</v>
       </c>
@@ -28161,7 +27902,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.05256000000003</v>
       </c>
-      <c r="Q292" s="22">
+      <c r="Q292">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>310.49704000000003</v>
       </c>
@@ -28230,7 +27971,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>176.12625</v>
       </c>
-      <c r="Q293" s="22">
+      <c r="Q293">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>321.19150400000001</v>
       </c>
@@ -28284,7 +28025,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>187.75595999999999</v>
       </c>
-      <c r="Q294" s="22">
+      <c r="Q294">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>333.57794199999995</v>
       </c>
@@ -28320,7 +28061,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q295" s="22">
+      <c r="Q295">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -28371,7 +28112,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q296" s="22">
+      <c r="Q296">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -28440,7 +28181,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>167.26527999999999</v>
       </c>
-      <c r="Q297" s="22">
+      <c r="Q297">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>321.39113599999996</v>
       </c>
@@ -28509,7 +28250,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.69925000000001</v>
       </c>
-      <c r="Q298" s="22">
+      <c r="Q298">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>295.66405400000002</v>
       </c>
@@ -28578,7 +28319,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>167.86751999999998</v>
       </c>
-      <c r="Q299" s="22">
+      <c r="Q299">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>313.59347500000001</v>
       </c>
@@ -28647,7 +28388,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>166.94886000000002</v>
       </c>
-      <c r="Q300" s="22">
+      <c r="Q300">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>312.52327200000002</v>
       </c>
@@ -28701,7 +28442,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>161.11428000000001</v>
       </c>
-      <c r="Q301" s="22">
+      <c r="Q301">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>296.31365399999999</v>
       </c>
@@ -28737,7 +28478,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q302" s="22">
+      <c r="Q302">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -28788,7 +28529,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q303" s="22">
+      <c r="Q303">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -28857,7 +28598,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>166.84704000000002</v>
       </c>
-      <c r="Q304" s="22">
+      <c r="Q304">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>285.85382800000002</v>
       </c>
@@ -28926,7 +28667,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>162.91368</v>
       </c>
-      <c r="Q305" s="22">
+      <c r="Q305">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>304.89558</v>
       </c>
@@ -28995,7 +28736,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.81745999999998</v>
       </c>
-      <c r="Q306" s="22">
+      <c r="Q306">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>323.44878</v>
       </c>
@@ -29064,7 +28805,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>166.2415</v>
       </c>
-      <c r="Q307" s="22">
+      <c r="Q307">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>313.97592599999996</v>
       </c>
@@ -29118,7 +28859,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>178.88210999999998</v>
       </c>
-      <c r="Q308" s="22">
+      <c r="Q308">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>322.32456000000008</v>
       </c>
@@ -29154,7 +28895,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q309" s="22">
+      <c r="Q309">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -29205,7 +28946,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q310" s="22">
+      <c r="Q310">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -29274,7 +29015,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.07984000000002</v>
       </c>
-      <c r="Q311" s="22">
+      <c r="Q311">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>304.164784</v>
       </c>
@@ -29343,7 +29084,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>166.84612999999999</v>
       </c>
-      <c r="Q312" s="22">
+      <c r="Q312">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>301.71225000000004</v>
       </c>
@@ -29412,7 +29153,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>168.48824999999999</v>
       </c>
-      <c r="Q313" s="22">
+      <c r="Q313">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>305.83855299999999</v>
       </c>
@@ -29481,7 +29222,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>167.232</v>
       </c>
-      <c r="Q314" s="22">
+      <c r="Q314">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>316.63989600000002</v>
       </c>
@@ -29535,7 +29276,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>162.35929999999999</v>
       </c>
-      <c r="Q315" s="22">
+      <c r="Q315">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>305.07240400000001</v>
       </c>
@@ -29571,7 +29312,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q316" s="22">
+      <c r="Q316">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -29622,7 +29363,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q317" s="22">
+      <c r="Q317">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -29691,7 +29432,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.25908999999999</v>
       </c>
-      <c r="Q318" s="22">
+      <c r="Q318">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>298.26641699999999</v>
       </c>
@@ -29760,7 +29501,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.63591</v>
       </c>
-      <c r="Q319" s="22">
+      <c r="Q319">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>322.010108</v>
       </c>
@@ -29829,7 +29570,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>166.66314</v>
       </c>
-      <c r="Q320" s="22">
+      <c r="Q320">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>312.790932</v>
       </c>
@@ -29898,7 +29639,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>167.71761999999998</v>
       </c>
-      <c r="Q321" s="22">
+      <c r="Q321">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>291.08916199999999</v>
       </c>
@@ -29952,7 +29693,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>177.2886</v>
       </c>
-      <c r="Q322" s="22">
+      <c r="Q322">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>323.24956800000001</v>
       </c>
@@ -29988,7 +29729,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q323" s="22">
+      <c r="Q323">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -30039,7 +29780,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q324" s="22">
+      <c r="Q324">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -30108,7 +29849,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>179.62924000000001</v>
       </c>
-      <c r="Q325" s="22">
+      <c r="Q325">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>302.07114699999994</v>
       </c>
@@ -30177,7 +29918,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>177.06597999999997</v>
       </c>
-      <c r="Q326" s="22">
+      <c r="Q326">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>300.09306600000002</v>
       </c>
@@ -30246,7 +29987,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>173.66711999999998</v>
       </c>
-      <c r="Q327" s="22">
+      <c r="Q327">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>287.95486800000003</v>
       </c>
@@ -30315,7 +30056,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>173.89279999999999</v>
       </c>
-      <c r="Q328" s="22">
+      <c r="Q328">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>295.51870000000002</v>
       </c>
@@ -30369,7 +30110,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>186.34390000000002</v>
       </c>
-      <c r="Q329" s="22">
+      <c r="Q329">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>301.72420799999998</v>
       </c>
@@ -30405,7 +30146,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q330" s="22">
+      <c r="Q330">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -30456,7 +30197,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q331" s="22">
+      <c r="Q331">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -30525,7 +30266,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>168.23688000000001</v>
       </c>
-      <c r="Q332" s="22">
+      <c r="Q332">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>309.88152500000001</v>
       </c>
@@ -30594,7 +30335,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.05707000000001</v>
       </c>
-      <c r="Q333" s="22">
+      <c r="Q333">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>309.78547500000002</v>
       </c>
@@ -30663,7 +30404,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.65360000000001</v>
       </c>
-      <c r="Q334" s="22">
+      <c r="Q334">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>307.22316000000001</v>
       </c>
@@ -30732,7 +30473,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.92624000000001</v>
       </c>
-      <c r="Q335" s="22">
+      <c r="Q335">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>301.06250999999997</v>
       </c>
@@ -30786,7 +30527,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>142.21912</v>
       </c>
-      <c r="Q336" s="22">
+      <c r="Q336">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>252.94338999999999</v>
       </c>
@@ -30822,7 +30563,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q337" s="22">
+      <c r="Q337">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -30873,7 +30614,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q338" s="22">
+      <c r="Q338">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -30942,7 +30683,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>174.90086000000002</v>
       </c>
-      <c r="Q339" s="22">
+      <c r="Q339">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>295.07328000000007</v>
       </c>
@@ -31011,7 +30752,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.1628</v>
       </c>
-      <c r="Q340" s="22">
+      <c r="Q340">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>297.44422500000002</v>
       </c>
@@ -31080,7 +30821,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.3158</v>
       </c>
-      <c r="Q341" s="22">
+      <c r="Q341">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>291.06596999999999</v>
       </c>
@@ -31149,7 +30890,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>172.03997999999999</v>
       </c>
-      <c r="Q342" s="22">
+      <c r="Q342">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>306.72128199999997</v>
       </c>
@@ -31203,7 +30944,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>174.96621999999999</v>
       </c>
-      <c r="Q343" s="22">
+      <c r="Q343">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>319.30719399999998</v>
       </c>
@@ -31239,7 +30980,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q344" s="22">
+      <c r="Q344">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -31290,7 +31031,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q345" s="22">
+      <c r="Q345">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -31359,7 +31100,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.98736</v>
       </c>
-      <c r="Q346" s="22">
+      <c r="Q346">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>307.20870000000002</v>
       </c>
@@ -31428,7 +31169,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.02438000000001</v>
       </c>
-      <c r="Q347" s="22">
+      <c r="Q347">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>313.41226</v>
       </c>
@@ -31497,7 +31238,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>168.60560000000001</v>
       </c>
-      <c r="Q348" s="22">
+      <c r="Q348">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>316.53751500000004</v>
       </c>
@@ -31566,7 +31307,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>174.75017</v>
       </c>
-      <c r="Q349" s="22">
+      <c r="Q349">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>321.35136</v>
       </c>
@@ -31620,7 +31361,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>168.95641000000001</v>
       </c>
-      <c r="Q350" s="22">
+      <c r="Q350">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>296.97055999999998</v>
       </c>
@@ -31656,7 +31397,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q351" s="22">
+      <c r="Q351">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -31707,7 +31448,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q352" s="22">
+      <c r="Q352">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -31776,7 +31517,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.51043999999999</v>
       </c>
-      <c r="Q353" s="22">
+      <c r="Q353">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>300.07872300000002</v>
       </c>
@@ -31845,7 +31586,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>176.49204</v>
       </c>
-      <c r="Q354" s="22">
+      <c r="Q354">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>323.35688700000003</v>
       </c>
@@ -31914,7 +31655,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>176.61847999999998</v>
       </c>
-      <c r="Q355" s="22">
+      <c r="Q355">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>318.32083499999999</v>
       </c>
@@ -31983,7 +31724,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>170.96970000000002</v>
       </c>
-      <c r="Q356" s="22">
+      <c r="Q356">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>310.43387200000001</v>
       </c>
@@ -32037,7 +31778,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>245.17151999999999</v>
       </c>
-      <c r="Q357" s="22">
+      <c r="Q357">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>427.386796</v>
       </c>
@@ -32073,7 +31814,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q358" s="22">
+      <c r="Q358">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -32124,7 +31865,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q359" s="22">
+      <c r="Q359">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -32193,7 +31934,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.96441000000002</v>
       </c>
-      <c r="Q360" s="22">
+      <c r="Q360">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>301.30976599999997</v>
       </c>
@@ -32262,7 +32003,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>169.32533000000001</v>
       </c>
-      <c r="Q361" s="22">
+      <c r="Q361">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>289.62086399999998</v>
       </c>
@@ -32331,7 +32072,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>173.31225000000001</v>
       </c>
-      <c r="Q362" s="22">
+      <c r="Q362">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>311.01734299999998</v>
       </c>
@@ -32400,7 +32141,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>171.55151999999998</v>
       </c>
-      <c r="Q363" s="22">
+      <c r="Q363">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>298.89822100000004</v>
       </c>
@@ -32454,7 +32195,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>154.04160000000002</v>
       </c>
-      <c r="Q364" s="22">
+      <c r="Q364">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>278.68044600000002</v>
       </c>
@@ -32490,7 +32231,7 @@
         <f>Tabla2[[#This Row],[cuba_fab_litros]]*Tabla2[[#This Row],[cuba_fab_prot_g_l]]/1000</f>
         <v>0</v>
       </c>
-      <c r="Q365" s="22">
+      <c r="Q365">
         <f>Tabla2[[#This Row],[queso_kg]]*Tabla2[[#This Row],[queso_est_pct]]/100</f>
         <v>0</v>
       </c>
@@ -32785,7 +32526,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -33350,6 +33090,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>